<commit_message>
alteracao da fila para banco de dados
</commit_message>
<xml_diff>
--- a/src/jmendes/excel_files/Robô Jmendes.xlsx
+++ b/src/jmendes/excel_files/Robô Jmendes.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29622"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29629"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67048" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78C1CE50-8FAE-42BE-9525-A28AB74907E2}"/>
+  <xr:revisionPtr revIDLastSave="67253" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{911C693C-5096-4043-B08A-535E755800A0}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="391">
   <si>
     <t>Data</t>
   </si>
@@ -85,6 +85,12 @@
     <t>Situação Final</t>
   </si>
   <si>
+    <t>08579947000291</t>
+  </si>
+  <si>
+    <t>08689024000292</t>
+  </si>
+  <si>
     <t>JMN</t>
   </si>
   <si>
@@ -109,16 +115,10 @@
     <t>Tarifa</t>
   </si>
   <si>
-    <t>08579947000291</t>
-  </si>
-  <si>
     <t>08579947000372</t>
   </si>
   <si>
     <t>Destinatário</t>
-  </si>
-  <si>
-    <t>08689024000292</t>
   </si>
   <si>
     <t xml:space="preserve">08689024000292 </t>
@@ -1116,9 +1116,6 @@
   </si>
   <si>
     <t>KRR7D11</t>
-  </si>
-  <si>
-    <t>levolog</t>
   </si>
   <si>
     <t>MATHEUS FELIPE DIAS</t>
@@ -2195,9 +2192,9 @@
     <col min="10" max="10" width="11.28515625" style="1" customWidth="1"/>
     <col min="11" max="11" width="23.140625" style="1" customWidth="1"/>
     <col min="12" max="12" width="20.42578125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" style="1" customWidth="1"/>
     <col min="14" max="14" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19" style="1" customWidth="1"/>
     <col min="20" max="20" width="15.85546875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2256,20 +2253,30 @@
       <c r="H2" s="59">
         <v>97</v>
       </c>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
+      <c r="I2" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J2" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K2" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" s="59" t="s">
+        <v>16</v>
+      </c>
       <c r="M2" s="60"/>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" s="62"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="59"/>
+      <c r="H3" s="59">
+        <v>97</v>
+      </c>
       <c r="I3" s="59"/>
       <c r="J3" s="59"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="61"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
       <c r="M3" s="60"/>
     </row>
     <row r="4" spans="1:20" s="50" customFormat="1">
@@ -2283,8 +2290,8 @@
       <c r="H4" s="59"/>
       <c r="I4" s="59"/>
       <c r="J4" s="59"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="61"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="59"/>
       <c r="N4" s="1"/>
       <c r="O4" s="59"/>
@@ -2305,8 +2312,8 @@
       <c r="H5" s="59"/>
       <c r="I5" s="59"/>
       <c r="J5" s="59"/>
-      <c r="K5" s="61"/>
-      <c r="L5" s="61"/>
+      <c r="K5" s="59"/>
+      <c r="L5" s="59"/>
       <c r="M5" s="60"/>
       <c r="N5" s="49"/>
       <c r="O5" s="49"/>
@@ -2318,17 +2325,17 @@
     </row>
     <row r="6" spans="1:20" s="50" customFormat="1">
       <c r="A6" s="62"/>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="62"/>
-      <c r="H6" s="62"/>
-      <c r="I6" s="62"/>
-      <c r="J6" s="62"/>
-      <c r="K6" s="62"/>
-      <c r="L6" s="62"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
       <c r="M6" s="60"/>
       <c r="N6" s="49"/>
       <c r="O6" s="1"/>
@@ -2340,93 +2347,63 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" s="62"/>
-      <c r="B7" s="62"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="62"/>
-      <c r="E7" s="62"/>
-      <c r="F7" s="62"/>
-      <c r="G7" s="62"/>
-      <c r="H7" s="62"/>
-      <c r="I7" s="62"/>
-      <c r="J7" s="62"/>
-      <c r="K7" s="62"/>
-      <c r="L7" s="62"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="59"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="59"/>
+      <c r="L7" s="59"/>
       <c r="M7" s="60"/>
       <c r="N7" s="49"/>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" s="62"/>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="62"/>
-      <c r="K8" s="62"/>
-      <c r="L8" s="62"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
       <c r="M8" s="60"/>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" s="62"/>
-      <c r="B9" s="62"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="62"/>
-      <c r="F9" s="62"/>
-      <c r="G9" s="62"/>
-      <c r="H9" s="62"/>
-      <c r="I9" s="62"/>
-      <c r="J9" s="62"/>
-      <c r="K9" s="62"/>
-      <c r="L9" s="62"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="59"/>
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
       <c r="M9" s="60"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="62"/>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
-      <c r="G10" s="62"/>
-      <c r="H10" s="62"/>
-      <c r="I10" s="62"/>
-      <c r="J10" s="62"/>
-      <c r="K10" s="62"/>
-      <c r="L10" s="62"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="59"/>
+      <c r="J10" s="59"/>
+      <c r="K10" s="59"/>
+      <c r="L10" s="59"/>
       <c r="M10" s="60"/>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" s="62"/>
-      <c r="B11" s="62"/>
-      <c r="C11" s="62"/>
-      <c r="D11" s="62"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
-      <c r="I11" s="62"/>
-      <c r="J11" s="62"/>
-      <c r="K11" s="62"/>
-      <c r="L11" s="62"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="59"/>
+      <c r="L11" s="59"/>
       <c r="M11" s="60"/>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" s="62"/>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="62"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="59"/>
+      <c r="L12" s="59"/>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" s="62"/>
@@ -2434,8 +2411,8 @@
       <c r="H13" s="59"/>
       <c r="I13" s="59"/>
       <c r="J13" s="59"/>
-      <c r="K13" s="61"/>
-      <c r="L13" s="61"/>
+      <c r="K13" s="59"/>
+      <c r="L13" s="59"/>
       <c r="N13" s="49"/>
     </row>
     <row r="14" spans="1:20">
@@ -2444,40 +2421,42 @@
       <c r="H14" s="59"/>
       <c r="I14" s="59"/>
       <c r="J14" s="59"/>
-      <c r="K14" s="61"/>
-      <c r="L14" s="61"/>
+      <c r="K14" s="59"/>
+      <c r="L14" s="59"/>
     </row>
     <row r="15" spans="1:20">
-      <c r="B15" s="59"/>
+      <c r="A15" s="62"/>
       <c r="G15" s="1"/>
       <c r="H15" s="59"/>
       <c r="I15" s="59"/>
       <c r="J15" s="59"/>
-      <c r="K15" s="61"/>
-      <c r="L15" s="61"/>
+      <c r="K15" s="59"/>
+      <c r="L15" s="59"/>
       <c r="M15" s="60"/>
     </row>
     <row r="16" spans="1:20">
+      <c r="A16" s="62"/>
       <c r="G16" s="1"/>
       <c r="H16" s="59"/>
       <c r="I16" s="59"/>
       <c r="J16" s="59"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
+      <c r="K16" s="59"/>
+      <c r="L16" s="59"/>
       <c r="M16" s="60"/>
     </row>
     <row r="17" spans="1:20">
+      <c r="A17" s="62"/>
       <c r="G17" s="1"/>
       <c r="H17" s="59"/>
       <c r="I17" s="59"/>
       <c r="J17" s="59"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="61"/>
+      <c r="K17" s="59"/>
+      <c r="L17" s="59"/>
       <c r="M17" s="60"/>
     </row>
     <row r="18" spans="1:20" s="50" customFormat="1">
-      <c r="A18" s="57"/>
-      <c r="B18" s="59"/>
+      <c r="A18" s="62"/>
+      <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -2486,8 +2465,8 @@
       <c r="H18" s="59"/>
       <c r="I18" s="59"/>
       <c r="J18" s="59"/>
-      <c r="K18" s="61"/>
-      <c r="L18" s="61"/>
+      <c r="K18" s="59"/>
+      <c r="L18" s="59"/>
       <c r="M18" s="60"/>
       <c r="N18" s="57"/>
       <c r="O18" s="57"/>
@@ -2498,40 +2477,42 @@
       <c r="T18" s="57"/>
     </row>
     <row r="19" spans="1:20">
-      <c r="B19" s="59"/>
+      <c r="A19" s="62"/>
       <c r="G19" s="1"/>
       <c r="H19" s="59"/>
       <c r="I19" s="59"/>
       <c r="J19" s="59"/>
-      <c r="K19" s="61"/>
-      <c r="L19" s="61"/>
+      <c r="K19" s="59"/>
+      <c r="L19" s="59"/>
     </row>
     <row r="20" spans="1:20">
+      <c r="A20" s="62"/>
       <c r="G20" s="1"/>
       <c r="H20" s="59"/>
       <c r="I20" s="59"/>
       <c r="J20" s="59"/>
-      <c r="K20" s="61"/>
-      <c r="L20" s="61"/>
+      <c r="K20" s="59"/>
+      <c r="L20" s="59"/>
       <c r="M20" s="60"/>
     </row>
     <row r="21" spans="1:20">
-      <c r="B21" s="59"/>
+      <c r="A21" s="62"/>
       <c r="G21" s="1"/>
       <c r="H21" s="59"/>
       <c r="I21" s="59"/>
       <c r="J21" s="59"/>
-      <c r="K21" s="61"/>
-      <c r="L21" s="61"/>
+      <c r="K21" s="59"/>
+      <c r="L21" s="59"/>
       <c r="M21" s="60"/>
     </row>
     <row r="22" spans="1:20">
+      <c r="A22" s="62"/>
       <c r="G22" s="1"/>
       <c r="H22" s="59"/>
       <c r="I22" s="59"/>
       <c r="J22" s="59"/>
-      <c r="K22" s="61"/>
-      <c r="L22" s="61"/>
+      <c r="K22" s="59"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="60"/>
     </row>
     <row r="23" spans="1:20">
@@ -2540,8 +2521,8 @@
       <c r="H23" s="59"/>
       <c r="I23" s="59"/>
       <c r="J23" s="59"/>
-      <c r="K23" s="61"/>
-      <c r="L23" s="61"/>
+      <c r="K23" s="59"/>
+      <c r="L23" s="59"/>
       <c r="M23" s="60"/>
     </row>
     <row r="24" spans="1:20">
@@ -2549,8 +2530,8 @@
       <c r="H24" s="59"/>
       <c r="I24" s="59"/>
       <c r="J24" s="59"/>
-      <c r="K24" s="61"/>
-      <c r="L24" s="61"/>
+      <c r="K24" s="59"/>
+      <c r="L24" s="59"/>
       <c r="M24" s="60"/>
     </row>
     <row r="25" spans="1:20">
@@ -2836,16 +2817,16 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="2:5">
@@ -2853,18 +2834,18 @@
         <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1">
         <v>32.5</v>
@@ -2879,21 +2860,21 @@
         <v>10</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>27</v>
@@ -2916,15 +2897,15 @@
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="13">
@@ -2947,7 +2928,7 @@
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>31</v>
@@ -5395,18 +5376,18 @@
         <v>358</v>
       </c>
       <c r="D174" s="32" t="s">
-        <v>359</v>
+        <v>42</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="15.75">
       <c r="A175" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B175" s="7">
         <v>757316245</v>
       </c>
       <c r="C175" s="29" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D175" s="32" t="s">
         <v>35</v>
@@ -5414,13 +5395,13 @@
     </row>
     <row r="176" spans="1:4" ht="15.75">
       <c r="A176" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B176" s="7">
         <v>757522487</v>
       </c>
       <c r="C176" s="29" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D176" s="32" t="s">
         <v>35</v>
@@ -5428,13 +5409,13 @@
     </row>
     <row r="177" spans="1:4" ht="15.75">
       <c r="A177" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B177" s="7">
         <v>757316286</v>
       </c>
       <c r="C177" s="29" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D177" s="32" t="s">
         <v>35</v>
@@ -5539,7 +5520,7 @@
       <c r="F2" s="35"/>
       <c r="G2" s="35"/>
       <c r="H2" s="51" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I2" s="52"/>
       <c r="J2" s="52"/>
@@ -5554,40 +5535,40 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="37" t="s">
+        <v>366</v>
+      </c>
+      <c r="B4" s="33" t="s">
         <v>367</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="C4" s="33" t="s">
         <v>368</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="D4" s="33" t="s">
         <v>369</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="E4" s="33" t="s">
         <v>370</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="G4" s="33" t="s">
         <v>371</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="H4" s="37" t="s">
+        <v>366</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>367</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>368</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>369</v>
+      </c>
+      <c r="L4" s="33" t="s">
+        <v>370</v>
+      </c>
+      <c r="M4" s="58" t="s">
         <v>372</v>
-      </c>
-      <c r="H4" s="37" t="s">
-        <v>367</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>368</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>370</v>
-      </c>
-      <c r="L4" s="33" t="s">
-        <v>371</v>
-      </c>
-      <c r="M4" s="58" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -5597,40 +5578,40 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="D6" s="50" t="s">
         <v>374</v>
       </c>
-      <c r="B6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="D6" s="50" t="s">
+      <c r="E6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="J6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="K6" s="50" t="s">
         <v>375</v>
       </c>
-      <c r="E6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="G6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>374</v>
-      </c>
-      <c r="I6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="J6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="K6" s="50" t="s">
-        <v>376</v>
-      </c>
       <c r="L6" s="32" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="M6" s="36" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -5640,41 +5621,41 @@
     </row>
     <row r="8" spans="1:13" ht="15.75">
       <c r="A8" s="43" t="s">
+        <v>376</v>
+      </c>
+      <c r="B8" s="44" t="s">
         <v>377</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="C8" s="44" t="s">
         <v>378</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="D8" s="44" t="s">
+        <v>378</v>
+      </c>
+      <c r="E8" s="44" t="s">
         <v>379</v>
-      </c>
-      <c r="D8" s="44" t="s">
-        <v>379</v>
-      </c>
-      <c r="E8" s="44" t="s">
-        <v>380</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44" t="s">
+        <v>380</v>
+      </c>
+      <c r="H8" s="43" t="s">
         <v>381</v>
       </c>
-      <c r="H8" s="43" t="s">
+      <c r="I8" s="44" t="s">
         <v>382</v>
       </c>
-      <c r="I8" s="44" t="s">
+      <c r="J8" s="44" t="s">
         <v>383</v>
       </c>
-      <c r="J8" s="44" t="s">
+      <c r="K8" s="44" t="s">
+        <v>383</v>
+      </c>
+      <c r="L8" s="44" t="s">
         <v>384</v>
       </c>
-      <c r="K8" s="44" t="s">
-        <v>384</v>
-      </c>
-      <c r="L8" s="44" t="s">
+      <c r="M8" s="44" t="s">
         <v>385</v>
-      </c>
-      <c r="M8" s="44" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5684,40 +5665,40 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="31" t="s">
+        <v>386</v>
+      </c>
+      <c r="B10" s="32" t="s">
         <v>387</v>
       </c>
-      <c r="B10" s="32" t="s">
-        <v>388</v>
-      </c>
       <c r="C10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="H10" s="31" t="s">
+        <v>386</v>
+      </c>
+      <c r="I10" s="32" t="s">
         <v>387</v>
       </c>
-      <c r="I10" s="32" t="s">
-        <v>388</v>
-      </c>
       <c r="J10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="K10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M10" s="36" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5727,40 +5708,40 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="K12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -5770,40 +5751,40 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="31" t="s">
+        <v>389</v>
+      </c>
+      <c r="B14" s="32" t="s">
         <v>390</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>391</v>
-      </c>
       <c r="C14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="H14" s="31" t="s">
+        <v>389</v>
+      </c>
+      <c r="I14" s="32" t="s">
         <v>390</v>
       </c>
-      <c r="I14" s="32" t="s">
-        <v>391</v>
-      </c>
       <c r="J14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="M14" s="36" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" spans="1:13">

</xml_diff>